<commit_message>
docs: one document per audit agenda item — EM26-28…32 (issued for approval)
- EM26-28 Contract Review Record (2025 university pilot; 2026 engagements)
- EM26-29 Software Requirements Specification (39 functional, 31 non-functional)
- EM26-30 Requirement Change Record (RC-2025-01 … RC-2026-07)
- EM26-31 Design and Development Record (8.3.2 → 8.3.6)
- EM26-32 Identification and Traceability Record (versions, traceability chain)
Evidence index updated. Public copy: clients as Client A–D.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
+++ b/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retrieve before the session" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evidence index'!$A$4:$F$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evidence index'!$A$4:$F$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Retrieve before the session'!$A$4:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -714,32 +714,32 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>02_Project_Plan</t>
+          <t>01_Contract_Review</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Jira board summary (project plan)</t>
+          <t>EM26-28 Contract Review Record</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>01_Contract_Review/EM26-28_Contract_Review_Record.docx</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Jira timeline</t>
+          <t>Jira board summary (project plan)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Jira board</t>
+          <t>Jira timeline</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -820,12 +820,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>SDLC project plan, roadmap and editions (Jun 2025 → Jul 2026)</t>
+          <t>Jira board</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -852,12 +852,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Scheduling review SCH-1.0 (May–Sep 2025)</t>
+          <t>SDLC project plan, roadmap and editions (Jun 2025 → Jul 2026)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -879,27 +879,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>EM26-12 Scheduling review (milestones, schedule risks)</t>
+          <t>Scheduling review SCH-1.0 (May–Sep 2025)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-12_Scheduling_Review.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tree/main/docs/qms/evidence-2026/12_Scheduling_Review</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>EM26-12 SDLC record (actual timeline, commits by month)</t>
+          <t>EM26-12 Scheduling review (milestones, schedule risks)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -926,12 +926,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-12_SDLC_Record.xlsx</t>
+          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-12_Scheduling_Review.docx</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tree/main/docs/qms/evidence-2026/12_Scheduling_Review</t>
         </is>
       </c>
     </row>
@@ -948,22 +948,22 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>EM26-22 Product roadmap 2025 → 2027 (timeline, plan vs actual, versions, forward plan)</t>
+          <t>EM26-12 SDLC record (actual timeline, commits by month)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-22_Product_Roadmap.xlsx</t>
+          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-12_SDLC_Record.xlsx</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -980,54 +980,54 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>EM26-23 Project Plan — EchoMind Enterprise</t>
+          <t>EM26-22 Product roadmap 2025 → 2027 (timeline, plan vs actual, versions, forward plan)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-23_Project_Plan_EchoMind_Enterprise.docx</t>
+          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-22_Product_Roadmap.xlsx</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client</t>
+          <t>02_Project_Plan</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Project documentation — EMD-02 (PO delay follow-up, August kick-off), EMD-12 (shipping confirmation and tracking)</t>
+          <t>EM26-23 Project Plan — EchoMind Enterprise</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2025-07 → 09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>02_Project_Plan/2026_EchoMind_Enterprise/EM26-23_Project_Plan_EchoMind_Enterprise.docx</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1044,12 +1044,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Deliverables review DR-1.0 — reviews held with the project lead</t>
+          <t>Project documentation — EMD-02 (PO delay follow-up, August kick-off), EMD-12 (shipping confirmation and tracking)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>2025-07 → 09</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1071,27 +1071,27 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-02 — client feedback</t>
+          <t>Deliverables review DR-1.0 — reviews held with the project lead</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-02_Requirements_Client_A_Client_B_Bahrain.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-03 — client feedback</t>
+          <t>Review record CR-2026-02 — client feedback</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-03_Conversation_assistance_v1_Kyutai_Unmute_stack.docx</t>
+          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-02_Requirements_Client_A_Client_B_Bahrain.docx</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-04 — client feedback</t>
+          <t>Review record CR-2026-03 — client feedback</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
+          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-03_Conversation_assistance_v1_Kyutai_Unmute_stack.docx</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-06 — client feedback</t>
+          <t>Review record CR-2026-04 — client feedback</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-06_Live_transcription.docx</t>
+          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-07 — client feedback</t>
+          <t>Review record CR-2026-06 — client feedback</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-07_Conversation_and_live_transcript_demonstration.docx</t>
+          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-06_Live_transcription.docx</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-09 — client feedback</t>
+          <t>Review record CR-2026-07 — client feedback</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-09_Document_creation.docx</t>
+          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-07_Conversation_and_live_transcript_demonstration.docx</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1263,59 +1263,59 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>EM26-27 Client Communication Log</t>
+          <t>Review record CR-2026-09 — client feedback</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>03_Communication_with_Client/EM26-27_Client_Communication_Log.xlsx</t>
+          <t>03_Communication_with_Client/2026_EchoMind_Enterprise/CR-2026-09_Document_creation.docx</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements</t>
+          <t>03_Communication_with_Client</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Requirements (ECH-QMS-010): fully offline on-premises AI system; BYOA pilot; acceptance by end-to-end test</t>
+          <t>EM26-27 Client Communication Log</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>03_Communication_with_Client/EM26-27_Client_Communication_Log.xlsx</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1332,12 +1332,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Acceptance criteria review ACC-1.0</t>
+          <t>Requirements (ECH-QMS-010): fully offline on-premises AI system; BYOA pilot; acceptance by end-to-end test</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2025-08-05</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1359,27 +1359,27 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>EM26-17 NFR record and monitoring (2025 finding #6)</t>
+          <t>Acceptance criteria review ACC-1.0</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025-09-04</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-17_NFR_Record_and_Monitoring.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1396,17 +1396,17 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 Functional requirements (39) with traceability</t>
+          <t>EM26-17 NFR record and monitoring (2025 finding #6)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-17_NFR_Record_and_Monitoring.docx</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>EM26-21 Non-functional requirements (31 + 9 from 2025) with measurements</t>
+          <t>EM26-20 Functional requirements (39) with traceability</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-21_Non_Functional_Requirements.xlsx</t>
+          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -1450,39 +1450,39 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements</t>
+          <t>04_Requirements</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>2025 change requests CR-2025-01 … 04 (lessons log)</t>
+          <t>EM26-21 Non-functional requirements (31 + 9 from 2025) with measurements</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>2025-05 → 09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-21_Non_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements</t>
+          <t>04_Requirements</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1492,22 +1492,22 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-03 — the client feedback that changed the requirement</t>
+          <t>EM26-29 Software Requirements Specification</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-03_Conversation_assistance_v1_Kyutai_Unmute_stack.docx</t>
+          <t>04_Requirements/EM26-29_Software_Requirements_Specification.docx</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1519,27 +1519,27 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-04 — the client feedback that changed the requirement</t>
+          <t>2025 change requests CR-2025-01 … 04 (lessons log)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-05 → 09</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-06 — the client feedback that changed the requirement</t>
+          <t>Review record CR-2026-03 — the client feedback that changed the requirement</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-06_Live_transcription.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-03_Conversation_assistance_v1_Kyutai_Unmute_stack.docx</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -1588,22 +1588,22 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>REG-07 Design and change register</t>
+          <t>Review record CR-2026-04 — the client feedback that changed the requirement</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/registers__REG-07_Design_and_Change_Register.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-07_Design_and_Change_Register.md</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -1620,22 +1620,22 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>SOP-06 Configuration and change management (significance criteria §6)</t>
+          <t>Review record CR-2026-06 — the client feedback that changed the requirement</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/procedures__SOP-06_Configuration_and_Change_Management.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-06_Live_transcription.docx</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>FRM-02 Change request (form)</t>
+          <t>REG-07 Design and change register</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1662,12 +1662,12 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/forms__FRM-02_Change_Request.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/registers__REG-07_Design_and_Change_Register.docx</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>QMS forms</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-07_Design_and_Change_Register.md</t>
         </is>
       </c>
     </row>
@@ -1684,118 +1684,118 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 › sheet ‘Requirement changes’ RC-2025-01 … RC-2026-07</t>
+          <t>SOP-06 Configuration and change management (significance criteria §6)</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/procedures__SOP-06_Configuration_and_Change_Management.docx</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development</t>
+          <t>05_Changes_to_Requirements</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Design and development process ECH-QMS-011 (inputs, outputs, controls); hardware BOM</t>
+          <t>FRM-02 Change request (form)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/forms__FRM-02_Change_Request.docx</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>QMS forms</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development</t>
+          <t>05_Changes_to_Requirements</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Architecture alignment workshop minutes MM-ECHO-2025-05</t>
+          <t>EM26-20 › sheet ‘Requirement changes’ RC-2025-01 … RC-2026-07</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development</t>
+          <t>05_Changes_to_Requirements</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-04 — design decision</t>
+          <t>EM26-30 Requirement Change Record</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
+          <t>05_Changes_to_Requirements/EM26-30_Requirement_Change_Record.docx</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1807,27 +1807,27 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-05 — design decision</t>
+          <t>Design and development process ECH-QMS-011 (inputs, outputs, controls); hardware BOM</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-05_Field_deployment_of_the_unit.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1839,27 +1839,27 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-08 — design decision</t>
+          <t>Architecture alignment workshop minutes MM-ECHO-2025-05</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-05-18</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-08_Group_discussions_Boardroom.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Review record SR-2026-01 — design decision</t>
+          <t>Review record CR-2026-04 — design decision</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/SR-2026-01_Security_and_defect_review_across_RAG_transcriptio.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -1908,22 +1908,22 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Design output — capabilities and how each module works</t>
+          <t>Review record CR-2026-05 — design decision</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-05_Field_deployment_of_the_unit.docx</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/CAPABILITIES.md</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -1940,22 +1940,22 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Design verification — dual-loop architecture, measured (QASC 2026)</t>
+          <t>Review record CR-2026-08 — design decision</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-08_Group_discussions_Boardroom.docx</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tree/main/docs/paper</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -1972,22 +1972,22 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>EM26-11 Deliverables review (Feb–Oct 2026)</t>
+          <t>Review record SR-2026-01 — design decision</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EM26-11_Deliverables_Review.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/SR-2026-01_Security_and_defect_review_across_RAG_transcriptio.docx</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -2004,150 +2004,150 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>SOP-05 Design and development control</t>
+          <t>Design output — capabilities and how each module works</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/procedures__SOP-05_Design_and_Development_Control.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/CAPABILITIES.md</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records</t>
+          <t>06_Design_and_Development</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — AJACE Deliverables Review EchoMind</t>
+          <t>Design verification — dual-loop architecture, measured (QASC 2026)</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tree/main/docs/paper</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records</t>
+          <t>06_Design_and_Development</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — AJACE Scheduling Review EchoMind</t>
+          <t>EM26-11 Deliverables review (Feb–Oct 2026)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EM26-11_Deliverables_Review.docx</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records</t>
+          <t>06_Design_and_Development</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — AJACE Acceptance Criteria Review EchoMind</t>
+          <t>SOP-05 Design and development control</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/procedures__SOP-05_Design_and_Development_Control.docx</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records</t>
+          <t>06_Design_and_Development</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — Meeting Minutes Architecture Workshop EchoMind</t>
+          <t>EM26-31 Design and Development Record</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>06_Design_and_Development/EM26-31_Design_and_Development_Record.docx</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — Meeting Minutes QA Sprint EchoMind</t>
+          <t>2025 review record / minutes — AJACE Deliverables Review EchoMind</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — Meeting Minutes Provider Review EchoMind</t>
+          <t>2025 review record / minutes — AJACE Scheduling Review EchoMind</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2223,27 +2223,27 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>2025-2026 All Review Records</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Review records DR-2025-01 … 15, CR-2026-01 … 09, SR-2026-01, RV-2026-01 … 08 (33)</t>
+          <t>2025 review record / minutes — AJACE Acceptance Criteria Review EchoMind</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>2025-05 → 2026-10</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records/2025-2026_All_Review_Records/Review_Records_all_33</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2255,27 +2255,27 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>EM26-18 Review feedback and action log (2025 finding #7)</t>
+          <t>2025 review record / minutes — Meeting Minutes Architecture Workshop EchoMind</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-18_Deliverable_Review_Feedback_and_Action_Log.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2287,34 +2287,34 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>EM26-19 Review feedback and action log (review cycle, version reviews, 75 actions)</t>
+          <t>2025 review record / minutes — Meeting Minutes QA Sprint EchoMind</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases</t>
+          <t>07_Review_Records</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-UI-Upload-001</t>
+          <t>2025 review record / minutes — Meeting Minutes Provider Review EchoMind</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2346,71 +2346,71 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases</t>
+          <t>07_Review_Records</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2025-2026 All Review Records</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-Stacks-002</t>
+          <t>Review records DR-2025-01 … 15, CR-2026-01 … 09, SR-2026-01, RV-2026-01 … 08 (33)</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-05 → 2026-10</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>07_Review_Records/2025-2026_All_Review_Records/Review_Records_all_33</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases</t>
+          <t>07_Review_Records</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-Transcribe-003</t>
+          <t>EM26-18 Review feedback and action log (2025 finding #7)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-18_Deliverable_Review_Feedback_and_Action_Log.docx</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases</t>
+          <t>07_Review_Records</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -2420,22 +2420,22 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>EM26-13 Acceptance criteria review</t>
+          <t>EM26-19 Review feedback and action log (review cycle, version reviews, 75 actions)</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-13_Acceptance_Criteria_Review.docx</t>
+          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
@@ -2447,27 +2447,27 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>13 acceptance test cases TC-EM-AUTH-101 … TC-EM-EVAL-114</t>
+          <t>2025 test case TC-EM-UI-Upload-001</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/Test_Cases</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2479,27 +2479,27 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>SOP-07 Verification, validation and testing</t>
+          <t>2025 test case TC-EM-Stacks-002</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/procedures__SOP-07_Verification_Validation_and_Testing.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2511,155 +2511,155 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>EM26-24 Test Plan — EchoMind Enterprise</t>
+          <t>2025 test case TC-EM-Transcribe-003</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-24_Test_Plan_EchoMind_Enterprise.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports</t>
+          <t>08_Test_Plan_and_Test_Cases</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Failed Functional Test QA-FAIL-01</t>
+          <t>EM26-13 Acceptance criteria review</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-13_Acceptance_Criteria_Review.docx</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports</t>
+          <t>08_Test_Plan_and_Test_Cases</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Defect Linking Jira DEF-2025-01</t>
+          <t>13 acceptance test cases TC-EM-AUTH-101 … TC-EM-EVAL-114</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/Test_Cases</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports</t>
+          <t>08_Test_Plan_and_Test_Cases</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Regression Testing Defects REG-2025-01</t>
+          <t>SOP-07 Verification, validation and testing</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/procedures__SOP-07_Verification_Validation_and_Testing.docx</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports</t>
+          <t>08_Test_Plan_and_Test_Cases</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — AJACE Test Failure EchoMind</t>
+          <t>EM26-24 Test Plan — EchoMind Enterprise</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-24_Test_Plan_EchoMind_Enterprise.docx</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2671,27 +2671,27 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Golden-question evaluation runs (24, 2026-07-29 → 09-22)</t>
+          <t>2025 test report — Failed Functional Test QA-FAIL-01</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 → 09-22</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Golden_Suite_Runs</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tree/main/eval/reports</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2703,27 +2703,27 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>EM26-15 Test summary report</t>
+          <t>2025 test report — Defect Linking Jira DEF-2025-01</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/EM26-15_Test_Summary_Report.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2735,27 +2735,27 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Acceptance test execution runs 1–4 (2026-10-06)</t>
+          <t>2025 test report — Regression Testing Defects REG-2025-01</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Execution_Records_run1-4</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2767,27 +2767,27 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Failure → defect → regression records QA-FAIL-2026-01 … 07, DEF-2026-01, REG-2026-01</t>
+          <t>2025 test report — AJACE Test Failure EchoMind</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Failure_Defect_Regression</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2804,61 +2804,61 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>CI runs and tickets</t>
+          <t>Golden-question evaluation runs (24, 2026-07-29 → 09-22)</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-07-29 → 09-22</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/CI_Runs_and_Tickets</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Golden_Suite_Runs</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tree/main/eval/reports</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Appliance identification ‘EchoMind – university’ unit; UPS tracking; versioned Git</t>
+          <t>EM26-15 Test summary report</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/EM26-15_Test_Summary_Report.docx</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>TC-EM-REL-106 Release identification test (pass, run 4)</t>
+          <t>Acceptance test execution runs 1–4 (2026-10-06)</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/TC-EM-REL-106_Release_identification_and_traceability.docx</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Execution_Records_run1-4</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
@@ -2890,7 +2890,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -2900,29 +2900,29 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>REG-08 Release and deployment register (versions v1.0.0 → v1.4.1, deployments)</t>
+          <t>Failure → defect → regression records QA-FAIL-2026-01 … 07, DEF-2026-01, REG-2026-01</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/registers__REG-08_Release_and_Deployment_Register.docx</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Failure_Defect_Regression</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-08_Release_and_Deployment_Register.md</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -2932,22 +2932,22 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Version tags v1.0.0 → v1.4.1 with their messages</t>
+          <t>CI runs and tickets</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/version_tags.txt</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/CI_Runs_and_Tickets</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tags</t>
+          <t>GitHub</t>
         </is>
       </c>
     </row>
@@ -2959,66 +2959,66 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 › sheet ‘Traceability’ (requirement → review → commit → version → test → release)</t>
+          <t>Appliance identification ‘EchoMind – university’ unit; UPS tracking; versioned Git</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Final release package approved and released (MM-2025-09-01)</t>
+          <t>TC-EM-REL-106 Release identification test (pass, run 4)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>2025-09-20</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/TC-EM-REL-106_Release_identification_and_traceability.docx</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -3028,29 +3028,29 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Release record (FRM-03) v1.4.0</t>
+          <t>REG-08 Release and deployment register (versions v1.0.0 → v1.4.1, deployments)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.0.docx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/registers__REG-08_Release_and_Deployment_Register.docx</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.0.md</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-08_Release_and_Deployment_Register.md</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -3060,29 +3060,29 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Release record (FRM-03) v1.4.1</t>
+          <t>Version tags v1.0.0 → v1.4.1 with their messages</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.1.docx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/version_tags.txt</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.1.md</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tags</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>CHANGELOG — one section per version</t>
+          <t>EM26-20 › sheet ‘Traceability’ (requirement → review → commit → version → test → release)</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3102,39 +3102,39 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/CHANGELOG.md</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/CHANGELOG.md</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>EM26-25 Release Notes v1.0.0 → v1.4.1</t>
+          <t>EM26-32 Identification and Traceability Record</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/EM26-25_Release_Notes_v1.0.0-v1.4.1.docx</t>
+          <t>10_Identification_and_Traceability/EM26-32_Identification_and_Traceability_Record.docx</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
@@ -3156,12 +3156,12 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — AJACE EchoMind Lessons Learned Log (May–Sep 2025)</t>
+          <t>Final release package approved and released (MM-2025-09-01)</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-09-20</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -3178,71 +3178,71 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — 16. AJACE_Lessons_Learnt_EchoMind</t>
+          <t>Release record (FRM-03) v1.4.0</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.0.docx</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.0.md</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — 16b. AJACE_Lessons_Learnt_Logbook_EchoMind</t>
+          <t>Release record (FRM-03) v1.4.1</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.1.docx</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.1.md</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -3252,29 +3252,29 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16 Lessons Learnt</t>
+          <t>CHANGELOG — one section per version</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt.docx</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/CHANGELOG.md</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/CHANGELOG.md</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -3284,22 +3284,22 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16b Lessons Learnt Logbook</t>
+          <t>EM26-25 Release Notes v1.0.0 → v1.4.1</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16b_Lessons_Learnt_Logbook.docx</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/EM26-25_Release_Notes_v1.0.0-v1.4.1.docx</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -3311,128 +3311,288 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16 Lessons Learnt Log</t>
+          <t>2025 lessons learnt — AJACE EchoMind Lessons Learned Log (May–Sep 2025)</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt_Log.xlsx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind</t>
+          <t>12_Lessons_Learnt</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Capabilities of the five modules</t>
+          <t>2025 lessons learnt — 16. AJACE_Lessons_Learnt_EchoMind</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind</t>
+          <t>12_Lessons_Learnt</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>QASC 2026 paper — EchoMind architecture and results</t>
+          <t>2025 lessons learnt — 16b. AJACE_Lessons_Learnt_Logbook_EchoMind</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>docs/paper</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>2026 lessons learnt — EM26-16 Lessons Learnt</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt.docx</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>2026 lessons learnt — EM26-16b Lessons Learnt Logbook</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16b_Lessons_Learnt_Logbook.docx</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>2026 lessons learnt — EM26-16 Lessons Learnt Log</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt_Log.xlsx</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
           <t>13_New_Use_Case_EchoMind</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>2026 EchoMind Enterprise</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Capabilities of the five modules</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>QASC 2026 paper — EchoMind architecture and results</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>docs/paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>EM26-26 New Use Cases — EchoMind Enterprise</t>
         </is>
       </c>
-      <c r="D95" s="4" t="inlineStr">
+      <c r="D100" s="4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E95" s="4" t="inlineStr">
+      <c r="E100" s="4" t="inlineStr">
         <is>
           <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EM26-26_New_Use_Cases_EchoMind_Enterprise.docx</t>
         </is>
       </c>
-      <c r="F95" s="4" t="inlineStr">
+      <c r="F100" s="4" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F95"/>
+  <autoFilter ref="A4:F100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: EM26-28 Development Side Contract Review — seven EchoMind development contracts
Replaces the earlier contract review record in the audit pack. Contract register and
FRM-11 review for each: university pilot (Aug 2025) and White edition (Oct 2025),
Client B conversation assistant (Dec 2025, frozen), Client A government project
(Feb 2026) and DoD FMR financial assistant (Mar 2026), Client D Document Studio
(Jun 2026), Client E IoT (Aug 2026, in evaluation). Issued for approval.

Public copy: clients as Client A–E.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
+++ b/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
@@ -724,7 +724,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>EM26-28 Contract Review Record</t>
+          <t>EM26-28 Development Side Contract Review</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>01_Contract_Review/EM26-28_Contract_Review_Record.docx</t>
+          <t>01_Contract_Review/EM26-28_Development_Side_Contract_Review.docx</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: client communication, requirement changes, design and development — revision 1.1
- EM26-27 Client Communication Record (new Word document) and log rev 1.1: every
  client and internal meeting Aug 2025 → Aug 2026 with feedback, decision, actions,
  requirements affected (FR/NFR) and where the meeting is recorded (EM26-19 / EM26-28)
- EM26-30 Requirement Change Record rev 1.1: reason, requester, meeting record,
  impact, decision, implementation (commit — version), verification; requirements
  added from internal reviews; requests not yet accepted
- EM26-31 Design and Development Record rev 1.1: design inputs from the FR/NFR
  registers; options evaluated and decisions (conversation, DoD FMR retrieval,
  hotspot, transcript accuracy, LLM speed, Silent Assistant, Boardroom, Document
  Studio) with the meeting where each was decided
Issued for approval. Public copy: clients as Client A–E.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
+++ b/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retrieve before the session" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evidence index'!$A$4:$F$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evidence index'!$A$4:$F$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Retrieve before the session'!$A$4:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1322,32 +1322,32 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements</t>
+          <t>03_Communication_with_Client</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Requirements (ECH-QMS-010): fully offline on-premises AI system; BYOA pilot; acceptance by end-to-end test</t>
+          <t>EM26-27 Client Communication Record (rev 1.1)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>03_Communication_with_Client/EM26-27_Client_Communication_Record.docx</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Acceptance criteria review ACC-1.0</t>
+          <t>Requirements (ECH-QMS-010): fully offline on-premises AI system; BYOA pilot; acceptance by end-to-end test</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2025-08-05</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1391,27 +1391,27 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>EM26-17 NFR record and monitoring (2025 finding #6)</t>
+          <t>Acceptance criteria review ACC-1.0</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025-09-04</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-17_NFR_Record_and_Monitoring.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1428,17 +1428,17 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 Functional requirements (39) with traceability</t>
+          <t>EM26-17 NFR record and monitoring (2025 finding #6)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-17_NFR_Record_and_Monitoring.docx</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>EM26-21 Non-functional requirements (31 + 9 from 2025) with measurements</t>
+          <t>EM26-20 Functional requirements (39) with traceability</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-21_Non_Functional_Requirements.xlsx</t>
+          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1492,54 +1492,54 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>EM26-29 Software Requirements Specification</t>
+          <t>EM26-21 Non-functional requirements (31 + 9 from 2025) with measurements</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>04_Requirements/EM26-29_Software_Requirements_Specification.docx</t>
+          <t>04_Requirements/2026_EchoMind_Enterprise/EM26-21_Non_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements</t>
+          <t>04_Requirements</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>2025 change requests CR-2025-01 … 04 (lessons log)</t>
+          <t>EM26-29 Software Requirements Specification</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>2025-05 → 09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>04_Requirements/EM26-29_Software_Requirements_Specification.docx</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1551,27 +1551,27 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-03 — the client feedback that changed the requirement</t>
+          <t>2025 change requests CR-2025-01 … 04 (lessons log)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-05 → 09</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-03_Conversation_assistance_v1_Kyutai_Unmute_stack.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-04 — the client feedback that changed the requirement</t>
+          <t>Review record CR-2026-03 — the client feedback that changed the requirement</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-03_Conversation_assistance_v1_Kyutai_Unmute_stack.docx</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-06 — the client feedback that changed the requirement</t>
+          <t>Review record CR-2026-04 — the client feedback that changed the requirement</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-06_Live_transcription.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -1652,22 +1652,22 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>REG-07 Design and change register</t>
+          <t>Review record CR-2026-06 — the client feedback that changed the requirement</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/registers__REG-07_Design_and_Change_Register.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/CR-2026-06_Live_transcription.docx</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-07_Design_and_Change_Register.md</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>SOP-06 Configuration and change management (significance criteria §6)</t>
+          <t>REG-07 Design and change register</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/procedures__SOP-06_Configuration_and_Change_Management.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/registers__REG-07_Design_and_Change_Register.docx</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-07_Design_and_Change_Register.md</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>FRM-02 Change request (form)</t>
+          <t>SOP-06 Configuration and change management (significance criteria §6)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1726,12 +1726,12 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/forms__FRM-02_Change_Request.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/procedures__SOP-06_Configuration_and_Change_Management.docx</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>QMS forms</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
@@ -1748,22 +1748,22 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 › sheet ‘Requirement changes’ RC-2025-01 … RC-2026-07</t>
+          <t>FRM-02 Change request (form)</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/forms__FRM-02_Change_Request.docx</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>QMS forms</t>
         </is>
       </c>
     </row>
@@ -1775,59 +1775,59 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>EM26-30 Requirement Change Record</t>
+          <t>EM26-20 › sheet ‘Requirement changes’ RC-2025-01 … RC-2026-07</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>05_Changes_to_Requirements/EM26-30_Requirement_Change_Record.docx</t>
+          <t>05_Changes_to_Requirements/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development</t>
+          <t>05_Changes_to_Requirements</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Design and development process ECH-QMS-011 (inputs, outputs, controls); hardware BOM</t>
+          <t>EM26-30 Requirement Change Record</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>05_Changes_to_Requirements/EM26-30_Requirement_Change_Record.docx</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Architecture alignment workshop minutes MM-ECHO-2025-05</t>
+          <t>Design and development process ECH-QMS-011 (inputs, outputs, controls); hardware BOM</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -1871,27 +1871,27 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-04 — design decision</t>
+          <t>Architecture alignment workshop minutes MM-ECHO-2025-05</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-05-18</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-05 — design decision</t>
+          <t>Review record CR-2026-04 — design decision</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-05_Field_deployment_of_the_unit.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-04_Conversation_assistance_v2_NVIDIA_PersonaPlex.docx</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Review record CR-2026-08 — design decision</t>
+          <t>Review record CR-2026-05 — design decision</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-08_Group_discussions_Boardroom.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-05_Field_deployment_of_the_unit.docx</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Review record SR-2026-01 — design decision</t>
+          <t>Review record CR-2026-08 — design decision</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/SR-2026-01_Security_and_defect_review_across_RAG_transcriptio.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CR-2026-08_Group_discussions_Boardroom.docx</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -2004,22 +2004,22 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Design output — capabilities and how each module works</t>
+          <t>Review record SR-2026-01 — design decision</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/SR-2026-01_Security_and_defect_review_across_RAG_transcriptio.docx</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/CAPABILITIES.md</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -2036,22 +2036,22 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Design verification — dual-loop architecture, measured (QASC 2026)</t>
+          <t>Design output — capabilities and how each module works</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tree/main/docs/paper</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/CAPABILITIES.md</t>
         </is>
       </c>
     </row>
@@ -2068,22 +2068,22 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>EM26-11 Deliverables review (Feb–Oct 2026)</t>
+          <t>Design verification — dual-loop architecture, measured (QASC 2026)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EM26-11_Deliverables_Review.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tree/main/docs/paper</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>SOP-05 Design and development control</t>
+          <t>EM26-11 Deliverables review (Feb–Oct 2026)</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/2026_EchoMind_Enterprise/procedures__SOP-05_Design_and_Development_Control.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/EM26-11_Deliverables_Review.docx</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -2127,59 +2127,59 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>EM26-31 Design and Development Record</t>
+          <t>SOP-05 Design and development control</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>06_Design_and_Development/EM26-31_Design_and_Development_Record.docx</t>
+          <t>06_Design_and_Development/2026_EchoMind_Enterprise/procedures__SOP-05_Design_and_Development_Control.docx</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records</t>
+          <t>06_Design_and_Development</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — AJACE Deliverables Review EchoMind</t>
+          <t>EM26-31 Design and Development Record</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>06_Design_and_Development/EM26-31_Design_and_Development_Record.docx</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — AJACE Scheduling Review EchoMind</t>
+          <t>2025 review record / minutes — AJACE Deliverables Review EchoMind</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — AJACE Acceptance Criteria Review EchoMind</t>
+          <t>2025 review record / minutes — AJACE Scheduling Review EchoMind</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — Meeting Minutes Architecture Workshop EchoMind</t>
+          <t>2025 review record / minutes — AJACE Acceptance Criteria Review EchoMind</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — Meeting Minutes QA Sprint EchoMind</t>
+          <t>2025 review record / minutes — Meeting Minutes Architecture Workshop EchoMind</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>2025 review record / minutes — Meeting Minutes Provider Review EchoMind</t>
+          <t>2025 review record / minutes — Meeting Minutes QA Sprint EchoMind</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2351,27 +2351,27 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>2025-2026 All Review Records</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Review records DR-2025-01 … 15, CR-2026-01 … 09, SR-2026-01, RV-2026-01 … 08 (33)</t>
+          <t>2025 review record / minutes — Meeting Minutes Provider Review EchoMind</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>2025-05 → 2026-10</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records/2025-2026_All_Review_Records/Review_Records_all_33</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Evidence Library</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2383,27 +2383,27 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025-2026 All Review Records</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>EM26-18 Review feedback and action log (2025 finding #7)</t>
+          <t>Review records DR-2025-01 … 15, CR-2026-01 … 09, SR-2026-01, RV-2026-01 … 08 (33)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025-05 → 2026-10</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-18_Deliverable_Review_Feedback_and_Action_Log.docx</t>
+          <t>07_Review_Records/2025-2026_All_Review_Records/Review_Records_all_33</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>Evidence Library</t>
         </is>
       </c>
     </row>
@@ -2420,17 +2420,17 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>EM26-19 Review feedback and action log (review cycle, version reviews, 75 actions)</t>
+          <t>EM26-18 Review feedback and action log (2025 finding #7)</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx</t>
+          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-18_Deliverable_Review_Feedback_and_Action_Log.docx</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -2442,32 +2442,32 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases</t>
+          <t>07_Review_Records</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-UI-Upload-001</t>
+          <t>EM26-19 Review feedback and action log (review cycle, version reviews, 75 actions)</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>07_Review_Records/2026_EchoMind_Enterprise/EM26-19_Deliverable_Review_Feedback_and_Action_Log.xlsx</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-Stacks-002</t>
+          <t>2025 test case TC-EM-UI-Upload-001</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-Transcribe-003</t>
+          <t>2025 test case TC-EM-Stacks-002</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2543,27 +2543,27 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>EM26-13 Acceptance criteria review</t>
+          <t>2025 test case TC-EM-Transcribe-003</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-13_Acceptance_Criteria_Review.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>13 acceptance test cases TC-EM-AUTH-101 … TC-EM-EVAL-114</t>
+          <t>EM26-13 Acceptance criteria review</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/Test_Cases</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-13_Acceptance_Criteria_Review.docx</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -2612,22 +2612,22 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>SOP-07 Verification, validation and testing</t>
+          <t>13 acceptance test cases TC-EM-AUTH-101 … TC-EM-EVAL-114</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/procedures__SOP-07_Verification_Validation_and_Testing.docx</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/Test_Cases</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -2644,54 +2644,54 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>EM26-24 Test Plan — EchoMind Enterprise</t>
+          <t>SOP-07 Verification, validation and testing</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-24_Test_Plan_EchoMind_Enterprise.docx</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/procedures__SOP-07_Verification_Validation_and_Testing.docx</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports</t>
+          <t>08_Test_Plan_and_Test_Cases</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Failed Functional Test QA-FAIL-01</t>
+          <t>EM26-24 Test Plan — EchoMind Enterprise</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-24_Test_Plan_EchoMind_Enterprise.docx</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Defect Linking Jira DEF-2025-01</t>
+          <t>2025 test report — Failed Functional Test QA-FAIL-01</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Regression Testing Defects REG-2025-01</t>
+          <t>2025 test report — Defect Linking Jira DEF-2025-01</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — AJACE Test Failure EchoMind</t>
+          <t>2025 test report — Regression Testing Defects REG-2025-01</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2799,27 +2799,27 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Golden-question evaluation runs (24, 2026-07-29 → 09-22)</t>
+          <t>2025 test report — AJACE Test Failure EchoMind</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 → 09-22</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Golden_Suite_Runs</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tree/main/eval/reports</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2836,22 +2836,22 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>EM26-15 Test summary report</t>
+          <t>Golden-question evaluation runs (24, 2026-07-29 → 09-22)</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-07-29 → 09-22</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/EM26-15_Test_Summary_Report.docx</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Golden_Suite_Runs</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tree/main/eval/reports</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Acceptance test execution runs 1–4 (2026-10-06)</t>
+          <t>EM26-15 Test summary report</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Execution_Records_run1-4</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/EM26-15_Test_Summary_Report.docx</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Failure → defect → regression records QA-FAIL-2026-01 … 07, DEF-2026-01, REG-2026-01</t>
+          <t>Acceptance test execution runs 1–4 (2026-10-06)</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Failure_Defect_Regression</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Execution_Records_run1-4</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
@@ -2932,54 +2932,54 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>CI runs and tickets</t>
+          <t>Failure → defect → regression records QA-FAIL-2026-01 … 07, DEF-2026-01, REG-2026-01</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/CI_Runs_and_Tickets</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Failure_Defect_Regression</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Appliance identification ‘EchoMind – university’ unit; UPS tracking; versioned Git</t>
+          <t>CI runs and tickets</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/CI_Runs_and_Tickets</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>GitHub</t>
         </is>
       </c>
     </row>
@@ -2991,27 +2991,27 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>TC-EM-REL-106 Release identification test (pass, run 4)</t>
+          <t>Appliance identification ‘EchoMind – university’ unit; UPS tracking; versioned Git</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/TC-EM-REL-106_Release_identification_and_traceability.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -3028,22 +3028,22 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>REG-08 Release and deployment register (versions v1.0.0 → v1.4.1, deployments)</t>
+          <t>TC-EM-REL-106 Release identification test (pass, run 4)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/registers__REG-08_Release_and_Deployment_Register.docx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/TC-EM-REL-106_Release_identification_and_traceability.docx</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-08_Release_and_Deployment_Register.md</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Version tags v1.0.0 → v1.4.1 with their messages</t>
+          <t>REG-08 Release and deployment register (versions v1.0.0 → v1.4.1, deployments)</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3070,12 +3070,12 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/version_tags.txt</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/registers__REG-08_Release_and_Deployment_Register.docx</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tags</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-08_Release_and_Deployment_Register.md</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 › sheet ‘Traceability’ (requirement → review → commit → version → test → release)</t>
+          <t>Version tags v1.0.0 → v1.4.1 with their messages</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3102,12 +3102,12 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/version_tags.txt</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tags</t>
         </is>
       </c>
     </row>
@@ -3119,59 +3119,59 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>EM26-32 Identification and Traceability Record</t>
+          <t>EM26-20 › sheet ‘Traceability’ (requirement → review → commit → version → test → release)</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/EM26-32_Identification_and_Traceability_Record.docx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Final release package approved and released (MM-2025-09-01)</t>
+          <t>EM26-32 Identification and Traceability Record</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>2025-09-20</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>10_Identification_and_Traceability/EM26-32_Identification_and_Traceability_Record.docx</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -3183,27 +3183,27 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Release record (FRM-03) v1.4.0</t>
+          <t>Final release package approved and released (MM-2025-09-01)</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2025-09-20</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.0.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.0.md</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Release record (FRM-03) v1.4.1</t>
+          <t>Release record (FRM-03) v1.4.0</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3230,12 +3230,12 @@
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.1.docx</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.0.docx</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.1.md</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.0.md</t>
         </is>
       </c>
     </row>
@@ -3252,22 +3252,22 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>CHANGELOG — one section per version</t>
+          <t>Release record (FRM-03) v1.4.1</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/CHANGELOG.md</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.1.docx</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/CHANGELOG.md</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.1.md</t>
         </is>
       </c>
     </row>
@@ -3284,54 +3284,54 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>EM26-25 Release Notes v1.0.0 → v1.4.1</t>
+          <t>CHANGELOG — one section per version</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/EM26-25_Release_Notes_v1.0.0-v1.4.1.docx</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/CHANGELOG.md</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/CHANGELOG.md</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — AJACE EchoMind Lessons Learned Log (May–Sep 2025)</t>
+          <t>EM26-25 Release Notes v1.0.0 → v1.4.1</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/EM26-25_Release_Notes_v1.0.0-v1.4.1.docx</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — 16. AJACE_Lessons_Learnt_EchoMind</t>
+          <t>2025 lessons learnt — AJACE EchoMind Lessons Learned Log (May–Sep 2025)</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — 16b. AJACE_Lessons_Learnt_Logbook_EchoMind</t>
+          <t>2025 lessons learnt — 16. AJACE_Lessons_Learnt_EchoMind</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -3407,27 +3407,27 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16 Lessons Learnt</t>
+          <t>2025 lessons learnt — 16b. AJACE_Lessons_Learnt_Logbook_EchoMind</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16b Lessons Learnt Logbook</t>
+          <t>2026 lessons learnt — EM26-16 Lessons Learnt</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16b_Lessons_Learnt_Logbook.docx</t>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt.docx</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16 Lessons Learnt Log</t>
+          <t>2026 lessons learnt — EM26-16b Lessons Learnt Logbook</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt_Log.xlsx</t>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16b_Lessons_Learnt_Logbook.docx</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
@@ -3498,7 +3498,7 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind</t>
+          <t>12_Lessons_Learnt</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -3508,22 +3508,22 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Capabilities of the five modules</t>
+          <t>2026 lessons learnt — EM26-16 Lessons Learnt Log</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt_Log.xlsx</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -3540,22 +3540,22 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>QASC 2026 paper — EchoMind architecture and results</t>
+          <t>Capabilities of the five modules</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>docs/paper</t>
+          <t>docs</t>
         </is>
       </c>
     </row>
@@ -3572,27 +3572,59 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
+          <t>QASC 2026 paper — EchoMind architecture and results</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>docs/paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
           <t>EM26-26 New Use Cases — EchoMind Enterprise</t>
         </is>
       </c>
-      <c r="D100" s="4" t="inlineStr">
+      <c r="D101" s="4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E100" s="4" t="inlineStr">
+      <c r="E101" s="4" t="inlineStr">
         <is>
           <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EM26-26_New_Use_Cases_EchoMind_Enterprise.docx</t>
         </is>
       </c>
-      <c r="F100" s="4" t="inlineStr">
+      <c r="F101" s="4" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F100"/>
+  <autoFilter ref="A4:F101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: development, review, test and release process; test execution register; release note per version
- EM26-33 Development, Review, Test and Release Process: roles (feature testing by
  the feature tester, feature review by the Project Lead and architect, repository
  care by the Lead Engineer), feature workflow, golden test rule, internal audit
  every three to four months in the second week (Nov 2026, Feb, Jun, Oct 2027)
- EM26-24 Test Plan rev 1.1: feature test and review steps; golden test rule
- EM26-34 Test Execution Register: 38 recorded test runs Sep 2025 → Oct 2026 with
  version, result, defect and evidence; counts per version
- Release notes v1.0.0 … v1.4.1: development window, commit range, requirements
  delivered, changes, version reviews, verification, known issues
Issued for approval. Public copy: clients as Client A–E.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
+++ b/docs/EchoMind_Audit_2026-10-14_Project2/00_Evidence_Index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retrieve before the session" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evidence index'!$A$4:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evidence index'!$A$4:$F$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Retrieve before the session'!$A$4:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2474,32 +2474,32 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases</t>
+          <t>07_Review_Records</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-UI-Upload-001</t>
+          <t>EM26-33 Development, Review, Test and Release Process</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>07_Review_Records/EM26-33_Development_Review_Test_and_Release_Process.docx</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-Stacks-002</t>
+          <t>2025 test case TC-EM-UI-Upload-001</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>2025 test case TC-EM-Transcribe-003</t>
+          <t>2025 test case TC-EM-Stacks-002</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2575,27 +2575,27 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>EM26-13 Acceptance criteria review</t>
+          <t>2025 test case TC-EM-Transcribe-003</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-13_Acceptance_Criteria_Review.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>13 acceptance test cases TC-EM-AUTH-101 … TC-EM-EVAL-114</t>
+          <t>EM26-13 Acceptance criteria review</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/Test_Cases</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-13_Acceptance_Criteria_Review.docx</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -2644,22 +2644,22 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>SOP-07 Verification, validation and testing</t>
+          <t>13 acceptance test cases TC-EM-AUTH-101 … TC-EM-EVAL-114</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/procedures__SOP-07_Verification_Validation_and_Testing.docx</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/Test_Cases</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -2676,54 +2676,54 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>EM26-24 Test Plan — EchoMind Enterprise</t>
+          <t>SOP-07 Verification, validation and testing</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-24_Test_Plan_EchoMind_Enterprise.docx</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/procedures__SOP-07_Verification_Validation_and_Testing.docx</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>QMS</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports</t>
+          <t>08_Test_Plan_and_Test_Cases</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Failed Functional Test QA-FAIL-01</t>
+          <t>EM26-24 Test Plan — EchoMind Enterprise</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>08_Test_Plan_and_Test_Cases/2026_EchoMind_Enterprise/EM26-24_Test_Plan_EchoMind_Enterprise.docx</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Defect Linking Jira DEF-2025-01</t>
+          <t>2025 test report — Failed Functional Test QA-FAIL-01</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — Regression Testing Defects REG-2025-01</t>
+          <t>2025 test report — Defect Linking Jira DEF-2025-01</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>2025 test report — AJACE Test Failure EchoMind</t>
+          <t>2025 test report — Regression Testing Defects REG-2025-01</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2831,27 +2831,27 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Golden-question evaluation runs (24, 2026-07-29 → 09-22)</t>
+          <t>2025 test report — AJACE Test Failure EchoMind</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 → 09-22</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Golden_Suite_Runs</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tree/main/eval/reports</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -2868,22 +2868,22 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>EM26-15 Test summary report</t>
+          <t>Golden-question evaluation runs (24, 2026-07-29 → 09-22)</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-07-29 → 09-22</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/EM26-15_Test_Summary_Report.docx</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Golden_Suite_Runs</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tree/main/eval/reports</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Acceptance test execution runs 1–4 (2026-10-06)</t>
+          <t>EM26-15 Test summary report</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Execution_Records_run1-4</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/EM26-15_Test_Summary_Report.docx</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Failure → defect → regression records QA-FAIL-2026-01 … 07, DEF-2026-01, REG-2026-01</t>
+          <t>Acceptance test execution runs 1–4 (2026-10-06)</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/Failure_Defect_Regression</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Execution_Records_run1-4</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
@@ -2964,86 +2964,86 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>CI runs and tickets</t>
+          <t>Failure → defect → regression records QA-FAIL-2026-01 … 07, DEF-2026-01, REG-2026-01</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>09_Test_Reports/2026_EchoMind_Enterprise/CI_Runs_and_Tickets</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/Failure_Defect_Regression</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Appliance identification ‘EchoMind – university’ unit; UPS tracking; versioned Git</t>
+          <t>CI runs and tickets</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>09_Test_Reports/2026_EchoMind_Enterprise/CI_Runs_and_Tickets</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>GitHub</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability</t>
+          <t>09_Test_Reports</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>TC-EM-REL-106 Release identification test (pass, run 4)</t>
+          <t>EM26-34 Test Execution Register</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/TC-EM-REL-106_Release_identification_and_traceability.docx</t>
+          <t>09_Test_Reports/EM26-34_Test_Execution_Register.xlsx</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -3055,27 +3055,27 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>REG-08 Release and deployment register (versions v1.0.0 → v1.4.1, deployments)</t>
+          <t>Appliance identification ‘EchoMind – university’ unit; UPS tracking; versioned Git</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/registers__REG-08_Release_and_Deployment_Register.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-08_Release_and_Deployment_Register.md</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -3092,22 +3092,22 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Version tags v1.0.0 → v1.4.1 with their messages</t>
+          <t>TC-EM-REL-106 Release identification test (pass, run 4)</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/version_tags.txt</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/TC-EM-REL-106_Release_identification_and_traceability.docx</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/tags</t>
+          <t>Evidence pack</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>EM26-20 › sheet ‘Traceability’ (requirement → review → commit → version → test → release)</t>
+          <t>REG-08 Release and deployment register (versions v1.0.0 → v1.4.1, deployments)</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/registers__REG-08_Release_and_Deployment_Register.docx</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Controlled copy</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/registers/REG-08_Release_and_Deployment_Register.md</t>
         </is>
       </c>
     </row>
@@ -3151,91 +3151,91 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>EM26-32 Identification and Traceability Record</t>
+          <t>Version tags v1.0.0 → v1.4.1 with their messages</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>10_Identification_and_Traceability/EM26-32_Identification_and_Traceability_Record.docx</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/version_tags.txt</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>https://github.com/RW2523/echomind-enterprise/tags</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Final release package approved and released (MM-2025-09-01)</t>
+          <t>EM26-20 › sheet ‘Traceability’ (requirement → review → commit → version → test → release)</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>2025-09-20</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>10_Identification_and_Traceability/2026_EchoMind_Enterprise/EM26-20_Functional_Requirements.xlsx</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>Controlled copy</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes</t>
+          <t>10_Identification_and_Traceability</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Release record (FRM-03) v1.4.0</t>
+          <t>EM26-32 Identification and Traceability Record</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.0.docx</t>
+          <t>10_Identification_and_Traceability/EM26-32_Identification_and_Traceability_Record.docx</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.0.md</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -3247,27 +3247,27 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>2026 EchoMind Enterprise</t>
+          <t>2025 University Project</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Release record (FRM-03) v1.4.1</t>
+          <t>Final release package approved and released (MM-2025-09-01)</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2025-09-20</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.1.docx</t>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.1.md</t>
+          <t>2025 evidence pack</t>
         </is>
       </c>
     </row>
@@ -3284,22 +3284,22 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>CHANGELOG — one section per version</t>
+          <t>Release record (FRM-03) v1.4.0</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/CHANGELOG.md</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.0.docx</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/RW2523/echomind-enterprise/blob/main/CHANGELOG.md</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.0.md</t>
         </is>
       </c>
     </row>
@@ -3316,125 +3316,125 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>EM26-25 Release Notes v1.0.0 → v1.4.1</t>
+          <t>Release record (FRM-03) v1.4.1</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>11_Release_Notes/2026_EchoMind_Enterprise/EM26-25_Release_Notes_v1.0.0-v1.4.1.docx</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/records__releases__2026-10-06_v1.4.1.docx</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/docs/qms/records/releases/2026-10-06_v1.4.1.md</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — AJACE EchoMind Lessons Learned Log (May–Sep 2025)</t>
+          <t>CHANGELOG — one section per version</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/CHANGELOG.md</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>https://github.com/RW2523/echomind-enterprise/blob/main/CHANGELOG.md</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — 16. AJACE_Lessons_Learnt_EchoMind</t>
+          <t>EM26-25 Release Notes v1.0.0 → v1.4.1</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>11_Release_Notes/2026_EchoMind_Enterprise/EM26-25_Release_Notes_v1.0.0-v1.4.1.docx</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>2025 University Project</t>
+          <t>2026 EchoMind Enterprise</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>2025 lessons learnt — 16b. AJACE_Lessons_Learnt_Logbook_EchoMind</t>
+          <t>Release note v1.0.0 (2026-02-05 → 2026-02-27, 82 commits)</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+          <t>11_Release_Notes/Release_Notes_per_Version/Release_Note_v1.0.0.docx</t>
         </is>
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>2025 evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -3444,29 +3444,29 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16 Lessons Learnt</t>
+          <t>Release note v1.1.0 (2026-03-03 → 2026-04-29, 32 commits)</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt.docx</t>
+          <t>11_Release_Notes/Release_Notes_per_Version/Release_Note_v1.1.0.docx</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -3476,29 +3476,29 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16b Lessons Learnt Logbook</t>
+          <t>Release note v1.2.0 (2026-05-27 → 2026-06-27, 44 commits)</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16b_Lessons_Learnt_Logbook.docx</t>
+          <t>11_Release_Notes/Release_Notes_per_Version/Release_Note_v1.2.0.docx</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -3508,29 +3508,29 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>2026 lessons learnt — EM26-16 Lessons Learnt Log</t>
+          <t>Release note v1.3.0 (2026-07-16 → 2026-08-16, 39 commits)</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt_Log.xlsx</t>
+          <t>11_Release_Notes/Release_Notes_per_Version/Release_Note_v1.3.0.docx</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Evidence pack</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
@@ -3540,29 +3540,29 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Capabilities of the five modules</t>
+          <t>Release note v1.4.0 (2026-09-04 → 2026-09-22, 9 commits)</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+          <t>11_Release_Notes/Release_Notes_per_Version/Release_Note_v1.4.0.docx</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>docs</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind</t>
+          <t>11_Release_Notes</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
@@ -3572,59 +3572,315 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>QASC 2026 paper — EchoMind architecture and results</t>
+          <t>Release note v1.4.1 (2026-09-22 → 2026-10-06, 10 commits)</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+          <t>11_Release_Notes/Release_Notes_per_Version/Release_Note_v1.4.1.docx</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>docs/paper</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>2025 University Project</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>2025 lessons learnt — AJACE EchoMind Lessons Learned Log (May–Sep 2025)</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>2025 evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>2025 University Project</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>2025 lessons learnt — 16. AJACE_Lessons_Learnt_EchoMind</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>2025 evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>2025 University Project</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>2025 lessons learnt — 16b. AJACE_Lessons_Learnt_Logbook_EchoMind</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>— held in the controlled copy (2025 original, names the 2025 customer)</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>2025 evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>2026 lessons learnt — EM26-16 Lessons Learnt</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt.docx</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>Evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>2026 lessons learnt — EM26-16b Lessons Learnt Logbook</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16b_Lessons_Learnt_Logbook.docx</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>Evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>2026 lessons learnt — EM26-16 Lessons Learnt Log</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>12_Lessons_Learnt/2026_EchoMind_Enterprise/EM26-16_Lessons_Learnt_Log.xlsx</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>Evidence pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
           <t>13_New_Use_Case_EchoMind</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t>2026 EchoMind Enterprise</t>
-        </is>
-      </c>
-      <c r="C101" s="4" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Capabilities of the five modules</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/CAPABILITIES.md</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>QASC 2026 paper — EchoMind architecture and results</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EchoMind_QASC2026_CameraReady_v4.pdf</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>docs/paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>13_New_Use_Case_EchoMind</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>2026 EchoMind Enterprise</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
         <is>
           <t>EM26-26 New Use Cases — EchoMind Enterprise</t>
         </is>
       </c>
-      <c r="D101" s="4" t="inlineStr">
+      <c r="D109" s="4" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E101" s="4" t="inlineStr">
+      <c r="E109" s="4" t="inlineStr">
         <is>
           <t>13_New_Use_Case_EchoMind/2026_EchoMind_Enterprise/EM26-26_New_Use_Cases_EchoMind_Enterprise.docx</t>
         </is>
       </c>
-      <c r="F101" s="4" t="inlineStr">
+      <c r="F109" s="4" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F101"/>
+  <autoFilter ref="A4:F109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>